<commit_message>
Update baseline model files; modify bergambacht, eemdijk, ijkdijk, and pernio runs
</commit_message>
<xml_diff>
--- a/baseline_models/bergambacht_v2_runs.xlsx
+++ b/baseline_models/bergambacht_v2_runs.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-6030" windowWidth="16440" windowHeight="28320" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3900" yWindow="345" windowWidth="12150" windowHeight="15585" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="runs" sheetId="1" state="visible" r:id="rId1"/>
@@ -55177,7 +55177,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-18 11:06:52</t>
+          <t>2026-05-28 11:53:34</t>
         </is>
       </c>
       <c r="D2" t="b">
@@ -55200,7 +55200,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-18 11:07:00</t>
+          <t>2026-05-28 11:53:44</t>
         </is>
       </c>
       <c r="D3" t="b">
@@ -55223,7 +55223,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-18 11:07:08</t>
+          <t>2026-05-28 11:53:55</t>
         </is>
       </c>
       <c r="D4" t="b">
@@ -55246,7 +55246,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-18 11:07:16</t>
+          <t>2026-05-28 11:54:08</t>
         </is>
       </c>
       <c r="D5" t="b">
@@ -55269,7 +55269,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-18 11:07:23</t>
+          <t>2026-05-28 11:54:17</t>
         </is>
       </c>
       <c r="D6" t="b">
@@ -55292,7 +55292,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-18 11:07:31</t>
+          <t>2026-05-28 11:54:28</t>
         </is>
       </c>
       <c r="D7" t="b">
@@ -55315,7 +55315,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-18 11:07:39</t>
+          <t>2026-05-28 11:54:37</t>
         </is>
       </c>
       <c r="D8" t="b">
@@ -55338,7 +55338,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-18 11:07:47</t>
+          <t>2026-05-28 11:54:47</t>
         </is>
       </c>
       <c r="D9" t="b">
@@ -55361,7 +55361,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-18 11:07:55</t>
+          <t>2026-05-28 11:54:56</t>
         </is>
       </c>
       <c r="D10" t="b">
@@ -55384,7 +55384,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-18 11:08:04</t>
+          <t>2026-05-28 11:55:05</t>
         </is>
       </c>
       <c r="D11" t="b">
@@ -55407,7 +55407,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-05-18 11:08:12</t>
+          <t>2026-05-28 11:55:16</t>
         </is>
       </c>
       <c r="D12" t="b">
@@ -55430,7 +55430,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-05-18 11:08:20</t>
+          <t>2026-05-28 11:55:26</t>
         </is>
       </c>
       <c r="D13" t="b">
@@ -55453,7 +55453,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-05-18 11:08:28</t>
+          <t>2026-05-28 11:55:36</t>
         </is>
       </c>
       <c r="D14" t="b">
@@ -55476,7 +55476,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-05-18 11:08:36</t>
+          <t>2026-05-28 11:55:46</t>
         </is>
       </c>
       <c r="D15" t="b">
@@ -55499,7 +55499,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-05-18 11:08:44</t>
+          <t>2026-05-28 11:55:56</t>
         </is>
       </c>
       <c r="D16" t="b">
@@ -55522,7 +55522,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-05-18 11:08:52</t>
+          <t>2026-05-28 11:56:05</t>
         </is>
       </c>
       <c r="D17" t="b">
@@ -55545,7 +55545,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-05-18 11:09:00</t>
+          <t>2026-05-28 11:56:15</t>
         </is>
       </c>
       <c r="D18" t="b">
@@ -55568,7 +55568,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-05-18 11:09:08</t>
+          <t>2026-05-28 11:56:24</t>
         </is>
       </c>
       <c r="D19" t="b">
@@ -55591,7 +55591,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-05-18 11:09:16</t>
+          <t>2026-05-28 11:56:35</t>
         </is>
       </c>
       <c r="D20" t="b">
@@ -55614,7 +55614,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-05-18 11:09:24</t>
+          <t>2026-05-28 11:56:45</t>
         </is>
       </c>
       <c r="D21" t="b">
@@ -55637,7 +55637,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-05-18 11:09:32</t>
+          <t>2026-05-28 11:56:54</t>
         </is>
       </c>
       <c r="D22" t="b">
@@ -55660,7 +55660,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-05-18 11:09:40</t>
+          <t>2026-05-28 11:57:04</t>
         </is>
       </c>
       <c r="D23" t="b">
@@ -55683,7 +55683,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-05-18 11:09:48</t>
+          <t>2026-05-28 11:57:13</t>
         </is>
       </c>
       <c r="D24" t="b">
@@ -55706,7 +55706,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-05-18 11:09:56</t>
+          <t>2026-05-28 11:57:24</t>
         </is>
       </c>
       <c r="D25" t="b">
@@ -55729,7 +55729,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-05-18 11:10:03</t>
+          <t>2026-05-28 11:57:34</t>
         </is>
       </c>
       <c r="D26" t="b">
@@ -55752,7 +55752,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-05-18 11:10:11</t>
+          <t>2026-05-28 11:57:44</t>
         </is>
       </c>
       <c r="D27" t="b">
@@ -55775,7 +55775,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-05-18 11:10:19</t>
+          <t>2026-05-28 11:57:54</t>
         </is>
       </c>
       <c r="D28" t="b">
@@ -55798,7 +55798,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-05-18 11:10:28</t>
+          <t>2026-05-28 11:58:04</t>
         </is>
       </c>
       <c r="D29" t="b">
@@ -55821,7 +55821,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-05-18 11:10:36</t>
+          <t>2026-05-28 11:58:13</t>
         </is>
       </c>
       <c r="D30" t="b">
@@ -55844,7 +55844,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-05-18 11:10:44</t>
+          <t>2026-05-28 11:58:23</t>
         </is>
       </c>
       <c r="D31" t="b">
@@ -55867,7 +55867,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-05-18 11:10:51</t>
+          <t>2026-05-28 11:58:32</t>
         </is>
       </c>
       <c r="D32" t="b">
@@ -55890,7 +55890,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-05-18 11:11:00</t>
+          <t>2026-05-28 11:58:43</t>
         </is>
       </c>
       <c r="D33" t="b">
@@ -55913,7 +55913,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-05-18 11:11:11</t>
+          <t>2026-05-28 11:58:54</t>
         </is>
       </c>
       <c r="D34" t="b">
@@ -55936,7 +55936,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-05-18 11:11:22</t>
+          <t>2026-05-28 11:59:06</t>
         </is>
       </c>
       <c r="D35" t="b">
@@ -55959,7 +55959,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-05-18 11:11:29</t>
+          <t>2026-05-28 11:59:15</t>
         </is>
       </c>
       <c r="D36" t="b">
@@ -55982,7 +55982,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-05-18 11:11:39</t>
+          <t>2026-05-28 11:59:26</t>
         </is>
       </c>
       <c r="D37" t="b">
@@ -56005,7 +56005,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-05-18 11:11:47</t>
+          <t>2026-05-28 11:59:36</t>
         </is>
       </c>
       <c r="D38" t="b">
@@ -56028,7 +56028,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-05-18 11:11:56</t>
+          <t>2026-05-28 11:59:48</t>
         </is>
       </c>
       <c r="D39" t="b">
@@ -56051,7 +56051,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-05-18 11:12:04</t>
+          <t>2026-05-28 11:59:57</t>
         </is>
       </c>
       <c r="D40" t="b">
@@ -56074,7 +56074,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-05-18 11:12:13</t>
+          <t>2026-05-28 12:00:08</t>
         </is>
       </c>
       <c r="D41" t="b">
@@ -56097,7 +56097,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-05-18 11:12:20</t>
+          <t>2026-05-28 12:00:17</t>
         </is>
       </c>
       <c r="D42" t="b">
@@ -56120,7 +56120,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-05-18 11:12:29</t>
+          <t>2026-05-28 12:00:29</t>
         </is>
       </c>
       <c r="D43" t="b">
@@ -56143,7 +56143,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-05-18 11:12:37</t>
+          <t>2026-05-28 12:00:37</t>
         </is>
       </c>
       <c r="D44" t="b">
@@ -56166,7 +56166,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-05-18 11:12:46</t>
+          <t>2026-05-28 12:00:48</t>
         </is>
       </c>
       <c r="D45" t="b">
@@ -56189,7 +56189,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-05-18 11:12:53</t>
+          <t>2026-05-28 12:00:57</t>
         </is>
       </c>
       <c r="D46" t="b">
@@ -56212,7 +56212,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-05-18 11:13:02</t>
+          <t>2026-05-28 12:01:09</t>
         </is>
       </c>
       <c r="D47" t="b">
@@ -56235,7 +56235,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-05-18 11:13:09</t>
+          <t>2026-05-28 12:01:17</t>
         </is>
       </c>
       <c r="D48" t="b">
@@ -56258,7 +56258,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-05-18 11:13:17</t>
+          <t>2026-05-28 12:01:26</t>
         </is>
       </c>
       <c r="D49" t="b">
@@ -56281,7 +56281,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-05-18 11:13:24</t>
+          <t>2026-05-28 12:01:34</t>
         </is>
       </c>
       <c r="D50" t="b">
@@ -56304,7 +56304,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-05-18 11:13:31</t>
+          <t>2026-05-28 12:01:43</t>
         </is>
       </c>
       <c r="D51" t="b">
@@ -56327,7 +56327,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-05-18 11:13:39</t>
+          <t>2026-05-28 12:01:52</t>
         </is>
       </c>
       <c r="D52" t="b">
@@ -56350,7 +56350,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-05-18 11:13:48</t>
+          <t>2026-05-28 12:02:04</t>
         </is>
       </c>
       <c r="D53" t="b">
@@ -56373,7 +56373,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-05-18 11:13:55</t>
+          <t>2026-05-28 12:02:13</t>
         </is>
       </c>
       <c r="D54" t="b">
@@ -56396,7 +56396,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-05-18 11:14:04</t>
+          <t>2026-05-28 12:02:24</t>
         </is>
       </c>
       <c r="D55" t="b">
@@ -56419,7 +56419,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-05-18 11:14:11</t>
+          <t>2026-05-28 12:02:32</t>
         </is>
       </c>
       <c r="D56" t="b">
@@ -56442,7 +56442,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-05-18 11:14:20</t>
+          <t>2026-05-28 12:02:43</t>
         </is>
       </c>
       <c r="D57" t="b">
@@ -56465,7 +56465,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-05-18 11:14:27</t>
+          <t>2026-05-28 12:02:54</t>
         </is>
       </c>
       <c r="D58" t="b">
@@ -56488,7 +56488,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-05-18 11:14:37</t>
+          <t>2026-05-28 12:03:05</t>
         </is>
       </c>
       <c r="D59" t="b">
@@ -56511,7 +56511,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-05-18 11:14:44</t>
+          <t>2026-05-28 12:03:14</t>
         </is>
       </c>
       <c r="D60" t="b">
@@ -56534,7 +56534,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-05-18 11:14:51</t>
+          <t>2026-05-28 12:03:23</t>
         </is>
       </c>
       <c r="D61" t="b">
@@ -56557,7 +56557,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2026-05-18 11:14:59</t>
+          <t>2026-05-28 12:03:33</t>
         </is>
       </c>
       <c r="D62" t="b">
@@ -56580,7 +56580,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2026-05-18 11:15:08</t>
+          <t>2026-05-28 12:03:45</t>
         </is>
       </c>
       <c r="D63" t="b">
@@ -56603,7 +56603,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-05-18 11:15:16</t>
+          <t>2026-05-28 12:03:55</t>
         </is>
       </c>
       <c r="D64" t="b">
@@ -56626,7 +56626,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2026-05-18 11:15:24</t>
+          <t>2026-05-28 12:04:05</t>
         </is>
       </c>
       <c r="D65" t="b">
@@ -56649,7 +56649,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2026-05-18 11:15:31</t>
+          <t>2026-05-28 12:04:14</t>
         </is>
       </c>
       <c r="D66" t="b">
@@ -56672,7 +56672,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2026-05-18 11:15:38</t>
+          <t>2026-05-28 12:04:24</t>
         </is>
       </c>
       <c r="D67" t="b">
@@ -56695,7 +56695,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-05-27 16:18:29</t>
+          <t>2026-05-28 12:04:34</t>
         </is>
       </c>
       <c r="D68" t="b">
@@ -56718,7 +56718,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026-05-27 16:18:37</t>
+          <t>2026-05-28 12:04:43</t>
         </is>
       </c>
       <c r="D69" t="b">
@@ -56741,7 +56741,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-05-27 16:18:45</t>
+          <t>2026-05-28 12:04:54</t>
         </is>
       </c>
       <c r="D70" t="b">
@@ -56764,7 +56764,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026-05-27 16:18:52</t>
+          <t>2026-05-28 12:05:04</t>
         </is>
       </c>
       <c r="D71" t="b">
@@ -56787,7 +56787,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026-05-27 16:19:00</t>
+          <t>2026-05-28 12:05:13</t>
         </is>
       </c>
       <c r="D72" t="b">
@@ -56810,7 +56810,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-05-27 16:19:07</t>
+          <t>2026-05-28 12:05:23</t>
         </is>
       </c>
       <c r="D73" t="b">
@@ -56833,7 +56833,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2026-05-27 16:19:14</t>
+          <t>2026-05-28 12:05:32</t>
         </is>
       </c>
       <c r="D74" t="b">
@@ -56856,7 +56856,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2026-05-27 16:19:22</t>
+          <t>2026-05-28 12:05:41</t>
         </is>
       </c>
       <c r="D75" t="b">
@@ -56879,7 +56879,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-05-27 16:19:29</t>
+          <t>2026-05-28 12:05:50</t>
         </is>
       </c>
       <c r="D76" t="b">
@@ -56902,7 +56902,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-05-27 16:19:38</t>
+          <t>2026-05-28 12:06:04</t>
         </is>
       </c>
       <c r="D77" t="b">
@@ -56925,7 +56925,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2026-05-27 16:19:45</t>
+          <t>2026-05-28 12:06:12</t>
         </is>
       </c>
       <c r="D78" t="b">
@@ -56948,7 +56948,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026-05-27 16:19:53</t>
+          <t>2026-05-28 12:06:22</t>
         </is>
       </c>
       <c r="D79" t="b">
@@ -56971,7 +56971,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026-05-27 16:20:01</t>
+          <t>2026-05-28 12:06:32</t>
         </is>
       </c>
       <c r="D80" t="b">
@@ -56994,7 +56994,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-05-27 16:20:09</t>
+          <t>2026-05-28 12:06:41</t>
         </is>
       </c>
       <c r="D81" t="b">
@@ -57017,7 +57017,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026-05-27 16:20:16</t>
+          <t>2026-05-28 12:06:50</t>
         </is>
       </c>
       <c r="D82" t="b">
@@ -57040,7 +57040,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-05-27 16:20:24</t>
+          <t>2026-05-28 12:07:00</t>
         </is>
       </c>
       <c r="D83" t="b">
@@ -57063,7 +57063,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-05-27 16:20:32</t>
+          <t>2026-05-28 12:07:11</t>
         </is>
       </c>
       <c r="D84" t="b">
@@ -57086,7 +57086,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2026-05-27 16:20:41</t>
+          <t>2026-05-28 12:07:22</t>
         </is>
       </c>
       <c r="D85" t="b">
@@ -57109,7 +57109,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-05-27 16:20:48</t>
+          <t>2026-05-28 12:07:32</t>
         </is>
       </c>
       <c r="D86" t="b">
@@ -57132,7 +57132,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-05-27 16:20:58</t>
+          <t>2026-05-28 12:07:44</t>
         </is>
       </c>
       <c r="D87" t="b">
@@ -57155,7 +57155,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-05-27 16:21:05</t>
+          <t>2026-05-28 12:07:56</t>
         </is>
       </c>
       <c r="D88" t="b">
@@ -57178,7 +57178,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2026-05-27 16:21:14</t>
+          <t>2026-05-28 12:08:07</t>
         </is>
       </c>
       <c r="D89" t="b">
@@ -57201,7 +57201,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2026-05-27 16:21:21</t>
+          <t>2026-05-28 12:08:18</t>
         </is>
       </c>
       <c r="D90" t="b">
@@ -57224,7 +57224,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2026-05-27 16:21:29</t>
+          <t>2026-05-28 12:08:29</t>
         </is>
       </c>
       <c r="D91" t="b">
@@ -57247,7 +57247,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-05-27 16:21:36</t>
+          <t>2026-05-28 12:08:38</t>
         </is>
       </c>
       <c r="D92" t="b">
@@ -57270,7 +57270,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-05-27 16:21:44</t>
+          <t>2026-05-28 12:08:48</t>
         </is>
       </c>
       <c r="D93" t="b">
@@ -57293,7 +57293,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-05-27 16:21:51</t>
+          <t>2026-05-28 12:08:59</t>
         </is>
       </c>
       <c r="D94" t="b">
@@ -57316,7 +57316,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2026-05-27 16:22:00</t>
+          <t>2026-05-28 12:09:12</t>
         </is>
       </c>
       <c r="D95" t="b">
@@ -57339,7 +57339,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2026-05-27 16:22:07</t>
+          <t>2026-05-28 12:09:22</t>
         </is>
       </c>
       <c r="D96" t="b">
@@ -57362,7 +57362,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2026-05-27 16:22:15</t>
+          <t>2026-05-28 12:09:31</t>
         </is>
       </c>
       <c r="D97" t="b">
@@ -57385,7 +57385,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2026-05-27 16:22:22</t>
+          <t>2026-05-28 12:09:41</t>
         </is>
       </c>
       <c r="D98" t="b">
@@ -57408,7 +57408,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2026-05-27 16:22:29</t>
+          <t>2026-05-28 12:09:50</t>
         </is>
       </c>
       <c r="D99" t="b">

</xml_diff>